<commit_message>
Add analytics workspace, AI engines, payslip dispatch, award chat, and healthcare demo pack updates
- Workforce analytics workspace (series, alerts/budget, leave impact, roster optimisation)
- AI engine catalogue and engine workspace UI
- Payslip generation and dispatch (SMTP / Outlook Graph / Resend) with dry-run mode
- Award chat routes with streaming
- Bulk shifts, leave parsing, employee enrichment domain logic
- Healthcare demo pack refresh incl. leave requests fixture
</commit_message>
<xml_diff>
--- a/mvp-documents/healthcare/04-timesheet-healthcare.xlsx
+++ b/mvp-documents/healthcare/04-timesheet-healthcare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1121,9 +1121,85 @@
         <v>sleepover 23:00 to 07:00</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>HC-007</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Sage Abdallah</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Registered Nurse</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Full-time</v>
+      </c>
+      <c r="E23" t="str">
+        <v>09/07/2026</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="G23" t="str">
+        <v>08:00</v>
+      </c>
+      <c r="H23" t="str">
+        <v>16:30</v>
+      </c>
+      <c r="I23">
+        <v>30</v>
+      </c>
+      <c r="J23">
+        <v>8</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Banksia Grove</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>HC-007</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Sage Abdallah</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Registered Nurse</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Full-time</v>
+      </c>
+      <c r="E24" t="str">
+        <v>11/07/2026</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Saturday</v>
+      </c>
+      <c r="G24" t="str">
+        <v>08:00</v>
+      </c>
+      <c r="H24" t="str">
+        <v>16:30</v>
+      </c>
+      <c r="I24">
+        <v>30</v>
+      </c>
+      <c r="J24">
+        <v>8</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Banksia Grove</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>